<commit_message>
Update budget: change Hardware Q1, add Training row and Notes sheet
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/samples/budget.xlsx
+++ b/samples/budget.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +446,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="C2" t="n">
         <v>1200</v>
@@ -487,6 +488,44 @@
       <c r="D4">
         <f>B4+C4</f>
         <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>150</v>
+      </c>
+      <c r="C5" t="n">
+        <v>200</v>
+      </c>
+      <c r="D5">
+        <f>B5+C5</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Revised after Q2 review</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add finance note on Notes sheet
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/samples/budget.xlsx
+++ b/samples/budget.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,6 +528,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Travel Q2 raised to 275 per finance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>